<commit_message>
Refactor AddMultipleMemberByExcel response handling and enhance InfoResponseParse for improved data parsing; update ExcelReader to support dynamic sheet data replacement; modify UserSteps for better status validation of responses.
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/Sample_File_Member.xlsx
+++ b/TestData/UploadFiles/Sample_File_Member.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30210"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ibz\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ibz\source\repos\RestAPI_AutomationFramework\TestData\UploadFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="3240" yWindow="3240" windowWidth="21585" windowHeight="11385"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="AddMultiMember_Response" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="191028"/>
 </workbook>
 </file>
 
@@ -74,7 +75,7 @@
     <t>No</t>
   </si>
   <si>
-    <t>sample2test2member@rovicare.com</t>
+    <t>sample3test3member@rovicare.com</t>
   </si>
   <si>
     <t>CEO</t>
@@ -86,113 +87,277 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>sample1test1member@rovicare.com</t>
+    <t>Member1</t>
+  </si>
+  <si>
+    <t>sample4test4member@rovicare.com</t>
+  </si>
+  <si>
+    <t>Sample2</t>
+  </si>
+  <si>
+    <t>Test2</t>
+  </si>
+  <si>
+    <t>Member2</t>
+  </si>
+  <si>
+    <t>Case Manager</t>
+  </si>
+  <si>
+    <t>sample5test5member@rovicare.com</t>
+  </si>
+  <si>
+    <t>Team Lead</t>
+  </si>
+  <si>
+    <t>MemberId</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="5">
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="1"/>
     </font>
     <font>
       <u/>
-      <sz val="10"/>
+      <sz val="11"/>
       <color theme="10"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Sheets">
+    <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr val="window"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4285F4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="EA4335"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="FBBC04"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="34A853"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="FF6D01"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="46BDC6"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -341,133 +506,246 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryRight="0" summaryBelow="0"/>
-  </sheetPr>
-  <sheetFormatPr defaultColWidth="14.42578" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="5" max="5" width="20.14063" customWidth="1"/>
-    <col min="11" max="11" width="31.14063" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.42578" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28516" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.14063" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.71094" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85547" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.57031" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.14063" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.85547" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.57031" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.42578" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.71094" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1">
-      <c r="A2">
+    <row r="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="4">
         <v>1111111111</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="4">
         <v>2222222222</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="4">
         <v>3333333333</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="D3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="4">
         <v>1111111111</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="4">
         <v>2222222222</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="4">
         <v>3333333333</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" t="s">
+      <c r="K3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="4" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1111112221</v>
+      </c>
+      <c r="G4" s="4">
+        <v>32323333333</v>
+      </c>
+      <c r="H4" s="4">
+        <v>3333333333</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="K2" r:id="rId1" display="sample2test2member@rovicare.com"/>
-    <hyperlink ref="K3" r:id="rId2" display="sample1test1member@rovicare.com"/>
+    <hyperlink ref="K2" r:id="rId1"/>
+    <hyperlink ref="K3" r:id="rId2"/>
   </hyperlinks>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13.28516" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.14063" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.57031" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.710938" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28516" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.28516" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.57031" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.85547" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.14063" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.855469" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.57031" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.28516" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.425781" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="2" customFormat="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update the excel retrival and update in the excel code updated
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/Sample_File_Member.xlsx
+++ b/TestData/UploadFiles/Sample_File_Member.xlsx
@@ -119,34 +119,34 @@
     <x:t>Status</x:t>
   </x:si>
   <x:si>
+    <x:t>32323333333</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1111111111</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>1111111111</x:t>
+    <x:t>1111112221</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Email already registered.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3333333333</x:t>
   </x:si>
   <x:si>
     <x:t>2222222222</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3333333333</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>Email already registered.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1111112221</x:t>
-  </x:si>
-  <x:si>
-    <x:t>32323333333</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -745,8 +745,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="K2" r:id="rId6"/>
-    <x:hyperlink ref="K3" r:id="rId7"/>
+    <x:hyperlink ref="K2" r:id="rId10"/>
+    <x:hyperlink ref="K3" r:id="rId11"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
@@ -826,7 +826,7 @@
     </x:row>
     <x:row r="2" spans="1:14">
       <x:c r="A2" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>12</x:v>
@@ -841,13 +841,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
         <x:v>16</x:v>
@@ -865,12 +865,12 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="N2" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:14">
       <x:c r="A3" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>20</x:v>
@@ -885,13 +885,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
         <x:v>16</x:v>
@@ -909,12 +909,12 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="N3" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:14">
       <x:c r="A4" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>24</x:v>
@@ -929,13 +929,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
         <x:v>40</x:v>
-      </x:c>
-      <x:c r="G4" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="H4" s="0" t="s">
-        <x:v>35</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
         <x:v>16</x:v>
@@ -953,7 +953,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="N4" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Refactor SaveAddMultiMemberByExcelResponseToExcel method to improve dynamic column handling; enhance LoginSteps for better response storage in Excel with specified columns.
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/Sample_File_Member.xlsx
+++ b/TestData/UploadFiles/Sample_File_Member.xlsx
@@ -745,8 +745,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="K2" r:id="rId10"/>
-    <x:hyperlink ref="K3" r:id="rId11"/>
+    <x:hyperlink ref="K2" r:id="rId8"/>
+    <x:hyperlink ref="K3" r:id="rId9"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
Refactor UserSteps to improve member status validation logic; enhance Excel handling in response methods for better data integrity and clarity.
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/Sample_File_Member.xlsx
+++ b/TestData/UploadFiles/Sample_File_Member.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30210"/>
+  <x:workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ibz\source\repos\RestAPI_AutomationFramework\TestData\UploadFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <x:workbookPr codeName="ThisWorkbook"/>
   <x:bookViews>
-    <x:workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="0" activeTab="1"/>
+    <x:workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="0" activeTab="0"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
     <x:t>CEO</x:t>
   </x:si>
   <x:si>
-    <x:t>Sample1</x:t>
+    <x:t>Sample23</x:t>
   </x:si>
   <x:si>
     <x:t>Test1</x:t>
@@ -92,13 +92,13 @@
     <x:t>Member1</x:t>
   </x:si>
   <x:si>
-    <x:t>sample4test4member@rovicare.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sample2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Test2</x:t>
+    <x:t>sample44test4member@rovicare.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sample26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Test2r</x:t>
   </x:si>
   <x:si>
     <x:t>Member2</x:t>
@@ -107,10 +107,7 @@
     <x:t>Case Manager</x:t>
   </x:si>
   <x:si>
-    <x:t>sample5test5member@rovicare.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Team Lead</x:t>
+    <x:t>sample55test5member@rovicare.com</x:t>
   </x:si>
   <x:si>
     <x:t>MemberId</x:t>
@@ -122,31 +119,34 @@
     <x:t>32323333333</x:t>
   </x:si>
   <x:si>
+    <x:t>1111112221</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2222222222</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
     <x:t>3</x:t>
   </x:si>
   <x:si>
+    <x:t>Email already registered.</x:t>
+  </x:si>
+  <x:si>
     <x:t>2</x:t>
   </x:si>
   <x:si>
+    <x:t>User exists in same organization</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3333333333</x:t>
+  </x:si>
+  <x:si>
     <x:t>1111111111</x:t>
   </x:si>
   <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
     <x:t>1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1111112221</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Email already registered.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3333333333</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2222222222</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -230,9 +230,8 @@
       </x:bottom>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="6">
+  <x:cellStyleXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -252,11 +251,11 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -270,9 +269,8 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
-  <x:cellStyles count="2">
+  <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <x:cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </x:cellStyles>
   <x:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
 </x:styleSheet>
@@ -740,7 +738,7 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="L4" s="7" t="s">
-        <x:v>29</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -761,7 +759,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:N4"/>
+  <x:dimension ref="A1:N13"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13.28516" style="0" bestFit="1" customWidth="1"/>
@@ -774,10 +772,10 @@
     <x:col min="8" max="8" width="14.57031" style="0" bestFit="1" customWidth="1"/>
     <x:col min="9" max="9" width="16.85547" style="0" bestFit="1" customWidth="1"/>
     <x:col min="10" max="10" width="19.14063" style="0" bestFit="1" customWidth="1"/>
-    <x:col min="11" max="11" width="5.855469" style="0" bestFit="1" customWidth="1"/>
+    <x:col min="11" max="11" width="33.71094" style="0" bestFit="1" customWidth="1"/>
     <x:col min="12" max="12" width="11.57031" style="0" bestFit="1" customWidth="1"/>
-    <x:col min="13" max="13" width="10.28516" style="0" bestFit="1" customWidth="1"/>
-    <x:col min="14" max="14" width="6.425781" style="0" bestFit="1" customWidth="1"/>
+    <x:col min="13" max="13" width="10.42578" style="0" bestFit="1" customWidth="1"/>
+    <x:col min="14" max="14" width="23" style="0" bestFit="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:14" s="2" customFormat="1">
@@ -818,15 +816,15 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="M1" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="N1" s="2" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="N1" s="2" t="s">
-        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:14">
       <x:c r="A2" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>12</x:v>
@@ -841,13 +839,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
         <x:v>16</x:v>
@@ -862,15 +860,15 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="N2" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:14">
       <x:c r="A3" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>20</x:v>
@@ -885,13 +883,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
         <x:v>16</x:v>
@@ -906,15 +904,15 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="M3" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="N3" s="0" t="s">
         <x:v>36</x:v>
-      </x:c>
-      <x:c r="N3" s="0" t="s">
-        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:14">
       <x:c r="A4" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>24</x:v>
@@ -929,13 +927,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
         <x:v>16</x:v>
@@ -947,14 +945,17 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="L4" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="M4" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="N4" s="0" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="N4" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:14">
+      <x:c r="K13" s="2"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
Refactored the excel data in the validation with response
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/Sample_File_Member.xlsx
+++ b/TestData/UploadFiles/Sample_File_Member.xlsx
@@ -14,6 +14,7 @@
   <x:sheets>
     <x:sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <x:sheet name="AddMultiMember_Response" sheetId="2" r:id="rId2"/>
+    <x:sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="191028"/>
@@ -59,13 +60,13 @@
     <x:t>Designation</x:t>
   </x:si>
   <x:si>
-    <x:t>Sample</x:t>
+    <x:t>friend</x:t>
   </x:si>
   <x:si>
     <x:t>Test</x:t>
   </x:si>
   <x:si>
-    <x:t>Member</x:t>
+    <x:t>LN</x:t>
   </x:si>
   <x:si>
     <x:t>Organization Admin</x:t>
@@ -77,37 +78,37 @@
     <x:t>No</x:t>
   </x:si>
   <x:si>
-    <x:t>sample3test3member@rovicare.com</x:t>
+    <x:t>LN1@rovicare.com</x:t>
   </x:si>
   <x:si>
     <x:t>CEO</x:t>
   </x:si>
   <x:si>
-    <x:t>Sample23</x:t>
+    <x:t>friend23</x:t>
   </x:si>
   <x:si>
     <x:t>Test1</x:t>
   </x:si>
   <x:si>
-    <x:t>Member1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>sample44test4member@rovicare.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sample26</x:t>
+    <x:t>LN1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LN2@rovicare.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>friend26</x:t>
   </x:si>
   <x:si>
     <x:t>Test2r</x:t>
   </x:si>
   <x:si>
-    <x:t>Member2</x:t>
+    <x:t>LN2</x:t>
   </x:si>
   <x:si>
     <x:t>Case Manager</x:t>
   </x:si>
   <x:si>
-    <x:t>sample55test5member@rovicare.com</x:t>
+    <x:t>LN3@rovicare.com</x:t>
   </x:si>
   <x:si>
     <x:t>MemberId</x:t>
@@ -125,16 +126,13 @@
     <x:t>2222222222</x:t>
   </x:si>
   <x:si>
+    <x:t>3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
     <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Email already registered.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2</x:t>
   </x:si>
   <x:si>
     <x:t>User exists in same organization</x:t>
@@ -156,7 +154,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="0" formatCode=""/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -183,13 +181,6 @@
       <x:color rgb="FF000000"/>
       <x:name val="Arial"/>
       <x:charset val="1"/>
-    </x:font>
-    <x:font>
-      <x:u/>
-      <x:sz val="11"/>
-      <x:color theme="10"/>
-      <x:name val="Calibri"/>
-      <x:scheme val="minor"/>
     </x:font>
     <x:font>
       <x:vertAlign val="baseline"/>
@@ -230,7 +221,7 @@
       </x:bottom>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="5">
+  <x:cellStyleXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
@@ -238,14 +229,11 @@
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -255,16 +243,12 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -658,7 +642,7 @@
       <x:c r="J2" s="7" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="K2" s="8" t="s">
+      <x:c r="K2" s="0" t="s">
         <x:v>18</x:v>
       </x:c>
       <x:c r="L2" s="7" t="s">
@@ -696,7 +680,7 @@
       <x:c r="J3" s="7" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="K3" s="8" t="s">
+      <x:c r="K3" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L3" s="7" t="s">
@@ -742,10 +726,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:hyperlinks>
-    <x:hyperlink ref="K2" r:id="rId8"/>
-    <x:hyperlink ref="K3" r:id="rId9"/>
-  </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -822,138 +802,6 @@
         <x:v>30</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:14">
-      <x:c r="A2" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D2" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F2" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G2" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H2" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="I2" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="J2" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="K2" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="L2" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M2" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="N2" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:14">
-      <x:c r="A3" s="0" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="I3" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="J3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="K3" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L3" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M3" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="N3" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:14">
-      <x:c r="A4" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="G4" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="H4" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="I4" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="J4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="K4" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="L4" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M4" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="N4" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-    </x:row>
     <x:row r="13" spans="1:14">
       <x:c r="K13" s="2"/>
     </x:row>
@@ -964,4 +812,197 @@
   <x:headerFooter/>
   <x:tableParts count="0"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:N4"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1" spans="1:14">
+      <x:c r="A1" s="0" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H1" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I1" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J1" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K1" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L1" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="M1" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="N1" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:14">
+      <x:c r="A2" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="K2" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L2" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="M2" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="N2" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:14">
+      <x:c r="A3" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="K3" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L3" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="M3" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="N3" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:14">
+      <x:c r="A4" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="K4" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="L4" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="M4" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="N4" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor Excel data handling in StoreInfo and AuthService to improve retrieval and response validation; enhance related methods for better consistency and error management.
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/Sample_File_Member.xlsx
+++ b/TestData/UploadFiles/Sample_File_Member.xlsx
@@ -120,31 +120,31 @@
     <x:t>32323333333</x:t>
   </x:si>
   <x:si>
+    <x:t>3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1111111111</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
     <x:t>1111112221</x:t>
   </x:si>
   <x:si>
+    <x:t>User exists in same organization</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3333333333</x:t>
+  </x:si>
+  <x:si>
     <x:t>2222222222</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>User exists in same organization</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3333333333</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1111111111</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -868,7 +868,7 @@
     </x:row>
     <x:row r="2" spans="1:14">
       <x:c r="A2" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>12</x:v>
@@ -883,13 +883,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
         <x:v>39</x:v>
-      </x:c>
-      <x:c r="G2" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H2" s="0" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
         <x:v>16</x:v>
@@ -904,7 +904,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="N2" s="0" t="s">
         <x:v>36</x:v>
@@ -912,7 +912,7 @@
     </x:row>
     <x:row r="3" spans="1:14">
       <x:c r="A3" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>20</x:v>
@@ -927,13 +927,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
         <x:v>39</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
         <x:v>16</x:v>
@@ -948,7 +948,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="M3" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="N3" s="0" t="s">
         <x:v>36</x:v>
@@ -956,7 +956,7 @@
     </x:row>
     <x:row r="4" spans="1:14">
       <x:c r="A4" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>24</x:v>
@@ -971,13 +971,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>31</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
         <x:v>16</x:v>
@@ -992,7 +992,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="M4" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="N4" s="0" t="s">
         <x:v>36</x:v>

</xml_diff>